<commit_message>
Whoops forgot some tests
</commit_message>
<xml_diff>
--- a/docs/lab02/Lab02_BBT_TCs_Form.xlsx
+++ b/docs/lab02/Lab02_BBT_TCs_Form.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10313"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BD252FB-8628-884B-A216-C72D93FD5A72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DB00940-C1E7-D046-9B4E-EA94E4AF8538}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="35840" windowHeight="22400" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -712,16 +712,16 @@
     <t>M...1234(256)</t>
   </si>
   <si>
-    <t>Save product does not throw exceptions</t>
-  </si>
-  <si>
-    <t>Now service has validator and throws exception</t>
-  </si>
-  <si>
     <t>YES</t>
   </si>
   <si>
     <t>Yes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validator doesn’t throw for max len of string being passed or null </t>
+  </si>
+  <si>
+    <t>Now validator has what it needs</t>
   </si>
 </sst>
 </file>
@@ -4232,35 +4232,35 @@
         <v>51</v>
       </c>
       <c r="C28" s="18">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="D28" s="20">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E28" s="20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F28" s="21" t="s">
+        <v>141</v>
+      </c>
+      <c r="G28" s="26" t="s">
+        <v>142</v>
+      </c>
+      <c r="H28" s="97" t="s">
         <v>139</v>
-      </c>
-      <c r="G28" s="26" t="s">
-        <v>140</v>
-      </c>
-      <c r="H28" s="97" t="s">
-        <v>141</v>
       </c>
       <c r="I28" s="98"/>
       <c r="J28" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K28" s="20">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L28" s="21">
         <v>0</v>
       </c>
       <c r="M28" s="25" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="N28" s="2">
         <v>10</v>

</xml_diff>